<commit_message>
Keep Gurobi, green levers, and hydrogen storage
</commit_message>
<xml_diff>
--- a/FinalModel_H2_without_additions/input_databases/h2_nl/technologies.xlsx
+++ b/FinalModel_H2_without_additions/input_databases/h2_nl/technologies.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F182"/>
+  <dimension ref="A1:F187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4443,37 +4443,39 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Battery</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Max hours</t>
+          <t>Long name</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr"/>
-      <c r="E176" t="n">
-        <v>4</v>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Underground hydrogen storage (salt cavern), addition</t>
+        </is>
       </c>
       <c r="F176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Long name</t>
+          <t>Sector</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Electrolyser on desalinated seawater (alternative water, outside the verdringingsreeks), lever</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -4481,19 +4483,19 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Sector</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Store</t>
         </is>
       </c>
       <c r="F178" t="inlineStr"/>
@@ -4501,19 +4503,23 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr"/>
+          <t>bus0</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>storage bus</t>
+        </is>
+      </c>
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Hydrogen</t>
         </is>
       </c>
       <c r="F179" t="inlineStr"/>
@@ -4521,52 +4527,36 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>bus0</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>main input</t>
-        </is>
-      </c>
+          <t>Start year</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr"/>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>Electricity</t>
-        </is>
+      <c r="E180" t="n">
+        <v>2030</v>
       </c>
       <c r="F180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>Battery</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>bus1</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>main output</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>Efficiency</t>
-        </is>
-      </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>Hydrogen</t>
-        </is>
+          <t>Max hours</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr"/>
+      <c r="D181" t="inlineStr"/>
+      <c r="E181" t="n">
+        <v>4</v>
       </c>
       <c r="F181" t="inlineStr"/>
     </row>
@@ -4578,15 +4568,127 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Start year</t>
+          <t>Long name</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr"/>
-      <c r="E182" t="n">
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Electrolyser on desalinated seawater (alternative water, outside the verdringingsreeks), lever</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" t="inlineStr"/>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr"/>
+      <c r="D184" t="inlineStr"/>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>bus0</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>main input</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>bus1</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>main output</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Start year</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr"/>
+      <c r="D187" t="inlineStr"/>
+      <c r="E187" t="n">
         <v>2030</v>
       </c>
-      <c r="F182" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4599,7 +4701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G173"/>
+  <dimension ref="A1:G178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8767,7 +8869,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -8777,26 +8879,26 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>€/kW</t>
+          <t>€/kWh</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>3666.7</v>
+        <v>0.9</v>
       </c>
       <c r="E169" t="n">
-        <v>2661.3</v>
+        <v>0.9</v>
       </c>
       <c r="F169" t="n">
-        <v>1923.1</v>
+        <v>0.85</v>
       </c>
       <c r="G169" t="n">
-        <v>1428.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -8806,26 +8908,26 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>€/kW</t>
+          <t>€/kWh</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>110</v>
+        <v>0.018</v>
       </c>
       <c r="E170" t="n">
-        <v>79.8</v>
+        <v>0.018</v>
       </c>
       <c r="F170" t="n">
-        <v>57.7</v>
+        <v>0.017</v>
       </c>
       <c r="G170" t="n">
-        <v>42.9</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -8854,7 +8956,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Electrolyser - seawater</t>
+          <t>H2 storage</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -8864,44 +8966,185 @@
       </c>
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E172" t="n">
-        <v>0.62</v>
+        <v>1</v>
       </c>
       <c r="F172" t="n">
-        <v>0.65</v>
+        <v>1</v>
       </c>
       <c r="G172" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
+          <t>H2 storage</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Lifetime</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>45</v>
+      </c>
+      <c r="E173" t="n">
+        <v>45</v>
+      </c>
+      <c r="F173" t="n">
+        <v>45</v>
+      </c>
+      <c r="G173" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
           <t>Electrolyser - seawater</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>€/kW</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>3666.7</v>
+      </c>
+      <c r="E174" t="n">
+        <v>2661.3</v>
+      </c>
+      <c r="F174" t="n">
+        <v>1923.1</v>
+      </c>
+      <c r="G174" t="n">
+        <v>1428.6</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>FOM</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>€/kW</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>110</v>
+      </c>
+      <c r="E175" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="F175" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="G175" t="n">
+        <v>42.9</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>VOM</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>€/kWh</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>0</v>
+      </c>
+      <c r="E176" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E177" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F177" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G177" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Electrolyser - seawater</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
         <is>
           <t>Lifetime</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
+      <c r="C178" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="D173" t="n">
+      <c r="D178" t="n">
         <v>25</v>
       </c>
-      <c r="E173" t="n">
+      <c r="E178" t="n">
         <v>25</v>
       </c>
-      <c r="F173" t="n">
+      <c r="F178" t="n">
         <v>25</v>
       </c>
-      <c r="G173" t="n">
+      <c r="G178" t="n">
         <v>25</v>
       </c>
     </row>

</xml_diff>